<commit_message>
add complete KTFL extraction project
</commit_message>
<xml_diff>
--- a/Output-Excel/395.xlsx
+++ b/Output-Excel/395.xlsx
@@ -9,7 +9,6 @@
   <sheets>
     <sheet name="Invoice Data" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Line Items" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Extraction Info" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -47,12 +46,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00145A32"/>
+        <fgColor rgb="00EBF3FB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="007F6000"/>
+        <fgColor rgb="00145A32"/>
       </patternFill>
     </fill>
   </fills>
@@ -73,9 +72,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -444,11 +441,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="65" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -476,12 +473,12 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Vendor</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>SAMATA TRANSPORT</t>
         </is>
@@ -500,14 +497,14 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Invoice Date</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-08-17</t>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>17.08.2026</t>
         </is>
       </c>
     </row>
@@ -517,164 +514,152 @@
           <t>PO Number</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>50-35586</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>All PO Numbers</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Vendor GSTIN</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>27AABCK0618A1Z7</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Handwritten References</t>
+          <t>HSN / SAC</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>50-35586, Die Shop freight o/w &amp; t/w charges, Provision taken on july-2026 = 233501, Bill month of Aug-2026 = 647621, 59174, 21/08/26, 12:20</t>
+          <t>00440262</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>GSTIN</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>27AABCK0618A127</t>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Vendor Code</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>80013</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>HSN/SAC</t>
+          <t>Currency</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>00440262</t>
+          <t>INR</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Vendor Code</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>80013</t>
-        </is>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Subtotal (Taxable Value)</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>88112</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Tax Code</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr"/>
+          <t>CGST</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Business Place</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Nagar - Pune Road, Near Garwa, Phalkemala, Tal - Shirur, Dist- Pune</t>
-        </is>
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>SGST</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Currency</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>INR</t>
-        </is>
+          <t>IGST</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Subtotal</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>88112</v>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Total Tax</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CGST</t>
+          <t>Invoice Total</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0</v>
+        <v>88112</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>SGST</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>0</v>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>GRN / Inward Number</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>59174</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>IGST</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>0</v>
+          <t>Handwritten References</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>50-35586</t>
+        </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Total Tax</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Invoice Total</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>88112</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Confidence %</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>0</v>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>AI Confidence %</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -691,7 +676,7 @@
   <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
@@ -700,32 +685,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Sl.No</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Item / Description</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Rate</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>HSN/SAC</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
@@ -753,72 +738,6 @@
       </c>
       <c r="F2" t="n">
         <v>88112</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="45" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>Field</t>
-        </is>
-      </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Extraction Method</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>LangChain + Ollama Qwen3-VL</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>HSN/SAC Rule</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Single invoice HSN/SAC applied to all items</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Handwriting Check</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Vision validation pass enabled</t>
-        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>